<commit_message>
feat: Add draw support to remote control and migrate rules to win=3, draw=1
</commit_message>
<xml_diff>
--- a/4학년피구대회일정.xlsx
+++ b/4학년피구대회일정.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\2026\학년협의\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\2026 송명신\피구대회\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B9403C-0192-4F07-80F6-1A3C717B1369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D512ADB-222F-4DA8-B7E9-711B6DB937D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="0" windowWidth="28215" windowHeight="15480" xr2:uid="{DD21F046-BAC6-4B5D-AC41-BB8291C46378}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD21F046-BAC6-4B5D-AC41-BB8291C46378}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -521,7 +521,7 @@
   </si>
   <si>
     <r>
-      <t>6반:</t>
+      <t>7반</t>
     </r>
     <r>
       <rPr>
@@ -532,506 +532,525 @@
         <charset val="129"/>
         <scheme val="minor"/>
       </rPr>
+      <t>:4반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>14반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:1반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>12반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:13반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>7반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:11반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>14반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:13반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2위:2위</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1위:1위</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>13반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:9반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>14반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:12반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:10반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>이순희</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>11반:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:12반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10반:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>11반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:7반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>8반:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>13반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>2반:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>11반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:9반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>14반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:6반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:4반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:10반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>14반:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>8반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>2반:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>심판명</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>횟수</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>3반:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10반</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6반</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>9반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>7반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:4반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>14반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:1반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>12반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:13반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>7반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:11반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>14반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:13반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>2위:2위</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1위:1위</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>13반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:9반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>14반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:12반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>4반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:10반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>이순희</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>11반:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>5반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>1반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:12반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>10반:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>11반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>5반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:7반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>8반:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>13반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>2반:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>11반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>1반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:9반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>14반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:6반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:4반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>5반</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:10반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>14반:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>8반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>2반:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>10반</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>심판명</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>횟수</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>3반:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>10반</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -1688,6 +1707,63 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1697,65 +1773,8 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2111,81 +2130,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
       <c r="D1" s="9"/>
-      <c r="J1" s="59" t="s">
+      <c r="J1" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="S1" s="59" t="s">
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="S1" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="59"/>
-      <c r="U1" s="59"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
       <c r="Z1" s="12"/>
-      <c r="AA1" s="59" t="s">
+      <c r="AA1" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="AB1" s="59"/>
-      <c r="AC1" s="59"/>
+      <c r="AB1" s="50"/>
+      <c r="AC1" s="50"/>
       <c r="AD1" s="9"/>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="58"/>
+      <c r="C2" s="60"/>
       <c r="D2" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="60" t="s">
+      <c r="E2" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="61"/>
-      <c r="G2" s="60" t="s">
+      <c r="F2" s="52"/>
+      <c r="G2" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="64"/>
+      <c r="H2" s="53"/>
       <c r="J2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="57" t="s">
+      <c r="K2" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="58"/>
+      <c r="L2" s="60"/>
       <c r="M2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="60" t="s">
+      <c r="N2" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="61"/>
-      <c r="P2" s="60" t="s">
+      <c r="O2" s="52"/>
+      <c r="P2" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="64"/>
+      <c r="Q2" s="53"/>
       <c r="S2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="T2" s="57" t="s">
+      <c r="T2" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="U2" s="58"/>
+      <c r="U2" s="60"/>
       <c r="V2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="W2" s="60" t="s">
+      <c r="W2" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="X2" s="61"/>
+      <c r="X2" s="52"/>
       <c r="Y2" s="26" t="s">
         <v>2</v>
       </c>
@@ -2193,28 +2212,28 @@
       <c r="AA2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="AB2" s="57" t="s">
+      <c r="AB2" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="AC2" s="58"/>
+      <c r="AC2" s="60"/>
       <c r="AD2" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="AE2" s="60" t="s">
+      <c r="AE2" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="AF2" s="61"/>
+      <c r="AF2" s="52"/>
       <c r="AG2" s="27" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:34" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
       <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
@@ -2224,54 +2243,54 @@
       <c r="G3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="51"/>
-      <c r="J3" s="55" t="s">
+      <c r="H3" s="64"/>
+      <c r="J3" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="54"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="58"/>
+      <c r="M3" s="61"/>
       <c r="N3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="50"/>
+      <c r="O3" s="58"/>
       <c r="P3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q3" s="51"/>
-      <c r="S3" s="55" t="s">
+      <c r="Q3" s="64"/>
+      <c r="S3" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="T3" s="50"/>
-      <c r="U3" s="50"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
       <c r="V3" s="62"/>
       <c r="W3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X3" s="50"/>
+      <c r="X3" s="58"/>
       <c r="Y3" s="7" t="s">
         <v>17</v>
       </c>
       <c r="Z3" s="14"/>
-      <c r="AA3" s="55" t="s">
+      <c r="AA3" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="AB3" s="50"/>
-      <c r="AC3" s="50"/>
-      <c r="AD3" s="50"/>
-      <c r="AE3" s="66" t="s">
+      <c r="AB3" s="58"/>
+      <c r="AC3" s="58"/>
+      <c r="AD3" s="58"/>
+      <c r="AE3" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="AF3" s="50"/>
+      <c r="AF3" s="58"/>
       <c r="AG3" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:34" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="56"/>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
+      <c r="A4" s="55"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
       <c r="E4" s="42" t="s">
         <v>35</v>
       </c>
@@ -2279,50 +2298,50 @@
         <v>36</v>
       </c>
       <c r="G4" s="43" t="s">
-        <v>52</v>
-      </c>
-      <c r="H4" s="51"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="50"/>
-      <c r="L4" s="50"/>
-      <c r="M4" s="54"/>
+        <v>51</v>
+      </c>
+      <c r="H4" s="64"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="61"/>
       <c r="N4" s="42" t="s">
-        <v>55</v>
-      </c>
-      <c r="O4" s="50"/>
+        <v>54</v>
+      </c>
+      <c r="O4" s="58"/>
       <c r="P4" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q4" s="51"/>
-      <c r="S4" s="56"/>
-      <c r="T4" s="50"/>
-      <c r="U4" s="50"/>
+        <v>64</v>
+      </c>
+      <c r="Q4" s="64"/>
+      <c r="S4" s="55"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="58"/>
       <c r="V4" s="63"/>
       <c r="W4" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="X4" s="50"/>
+        <v>46</v>
+      </c>
+      <c r="X4" s="58"/>
       <c r="Y4" s="7" t="s">
         <v>18</v>
       </c>
       <c r="Z4" s="14"/>
-      <c r="AA4" s="56"/>
-      <c r="AB4" s="50"/>
-      <c r="AC4" s="50"/>
-      <c r="AD4" s="50"/>
+      <c r="AA4" s="55"/>
+      <c r="AB4" s="58"/>
+      <c r="AC4" s="58"/>
+      <c r="AD4" s="58"/>
       <c r="AE4" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="AF4" s="50"/>
+        <v>67</v>
+      </c>
+      <c r="AF4" s="58"/>
       <c r="AG4" s="6"/>
     </row>
     <row r="5" spans="1:34" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="55" t="s">
+      <c r="A5" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
       <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
@@ -2332,50 +2351,50 @@
       <c r="G5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="51"/>
-      <c r="J5" s="55" t="s">
+      <c r="H5" s="64"/>
+      <c r="J5" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="K5" s="50"/>
-      <c r="L5" s="50"/>
-      <c r="M5" s="54"/>
+      <c r="K5" s="58"/>
+      <c r="L5" s="58"/>
+      <c r="M5" s="61"/>
       <c r="N5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O5" s="50"/>
+      <c r="O5" s="58"/>
       <c r="P5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q5" s="51"/>
-      <c r="S5" s="55" t="s">
+      <c r="Q5" s="64"/>
+      <c r="S5" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="T5" s="50"/>
-      <c r="U5" s="50"/>
+      <c r="T5" s="58"/>
+      <c r="U5" s="58"/>
       <c r="V5" s="62"/>
       <c r="W5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="X5" s="50"/>
+      <c r="X5" s="58"/>
       <c r="Y5" s="7"/>
       <c r="Z5" s="14"/>
-      <c r="AA5" s="55" t="s">
+      <c r="AA5" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="AB5" s="50"/>
-      <c r="AC5" s="50"/>
-      <c r="AD5" s="50"/>
+      <c r="AB5" s="58"/>
+      <c r="AC5" s="58"/>
+      <c r="AD5" s="58"/>
       <c r="AE5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="AF5" s="50"/>
+      <c r="AF5" s="58"/>
       <c r="AG5" s="5"/>
     </row>
     <row r="6" spans="1:34" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="56"/>
-      <c r="B6" s="50"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
+      <c r="A6" s="55"/>
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
       <c r="E6" s="10" t="s">
         <v>32</v>
       </c>
@@ -2383,253 +2402,253 @@
         <v>37</v>
       </c>
       <c r="G6" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="H6" s="51"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="50"/>
-      <c r="L6" s="50"/>
-      <c r="M6" s="54"/>
+        <v>52</v>
+      </c>
+      <c r="H6" s="64"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="58"/>
+      <c r="L6" s="58"/>
+      <c r="M6" s="61"/>
       <c r="N6" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="O6" s="50"/>
+      <c r="O6" s="58"/>
       <c r="P6" s="43" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q6" s="51"/>
-      <c r="S6" s="56"/>
-      <c r="T6" s="50"/>
-      <c r="U6" s="50"/>
+        <v>63</v>
+      </c>
+      <c r="Q6" s="64"/>
+      <c r="S6" s="55"/>
+      <c r="T6" s="58"/>
+      <c r="U6" s="58"/>
       <c r="V6" s="63"/>
       <c r="W6" s="43" t="s">
-        <v>57</v>
-      </c>
-      <c r="X6" s="50"/>
+        <v>56</v>
+      </c>
+      <c r="X6" s="58"/>
       <c r="Y6" s="8"/>
       <c r="Z6" s="14"/>
-      <c r="AA6" s="56"/>
-      <c r="AB6" s="50"/>
-      <c r="AC6" s="50"/>
-      <c r="AD6" s="50"/>
+      <c r="AA6" s="55"/>
+      <c r="AB6" s="58"/>
+      <c r="AC6" s="58"/>
+      <c r="AD6" s="58"/>
       <c r="AE6" s="43" t="s">
-        <v>49</v>
-      </c>
-      <c r="AF6" s="50"/>
+        <v>48</v>
+      </c>
+      <c r="AF6" s="58"/>
       <c r="AG6" s="6"/>
     </row>
     <row r="7" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="50"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
-      <c r="E7" s="47" t="s">
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="48"/>
+      <c r="F7" s="67"/>
       <c r="G7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H7" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="55" t="s">
+      <c r="J7" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="50"/>
-      <c r="L7" s="50"/>
-      <c r="M7" s="54"/>
+      <c r="K7" s="58"/>
+      <c r="L7" s="58"/>
+      <c r="M7" s="61"/>
       <c r="N7" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="O7" s="50"/>
+      <c r="O7" s="58"/>
       <c r="P7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="Q7" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="S7" s="55" t="s">
+      <c r="S7" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="T7" s="50"/>
-      <c r="U7" s="50"/>
+      <c r="T7" s="58"/>
+      <c r="U7" s="58"/>
       <c r="V7" s="62"/>
       <c r="W7" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="X7" s="50"/>
+      <c r="X7" s="58"/>
       <c r="Y7" s="7"/>
       <c r="Z7" s="15"/>
-      <c r="AA7" s="55" t="s">
+      <c r="AA7" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="AB7" s="50"/>
-      <c r="AC7" s="50"/>
-      <c r="AD7" s="50"/>
+      <c r="AB7" s="58"/>
+      <c r="AC7" s="58"/>
+      <c r="AD7" s="58"/>
       <c r="AE7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="AF7" s="50"/>
+      <c r="AF7" s="58"/>
       <c r="AG7" s="5"/>
     </row>
     <row r="8" spans="1:34" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="56"/>
-      <c r="B8" s="50"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="47" t="s">
+      <c r="A8" s="55"/>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="66" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="48"/>
+      <c r="F8" s="67"/>
       <c r="G8" s="28" t="s">
         <v>38</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="J8" s="56"/>
-      <c r="K8" s="50"/>
-      <c r="L8" s="50"/>
-      <c r="M8" s="54"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="58"/>
+      <c r="L8" s="58"/>
+      <c r="M8" s="61"/>
       <c r="N8" s="42" t="s">
-        <v>60</v>
-      </c>
-      <c r="O8" s="50"/>
+        <v>59</v>
+      </c>
+      <c r="O8" s="58"/>
       <c r="P8" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="Q8" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="S8" s="56"/>
-      <c r="T8" s="50"/>
-      <c r="U8" s="50"/>
+      <c r="Q8" s="43" t="s">
+        <v>71</v>
+      </c>
+      <c r="S8" s="55"/>
+      <c r="T8" s="58"/>
+      <c r="U8" s="58"/>
       <c r="V8" s="63"/>
       <c r="W8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="X8" s="50"/>
+      <c r="X8" s="58"/>
       <c r="Y8" s="8"/>
       <c r="Z8" s="16"/>
-      <c r="AA8" s="56"/>
-      <c r="AB8" s="50"/>
-      <c r="AC8" s="50"/>
-      <c r="AD8" s="50"/>
+      <c r="AA8" s="55"/>
+      <c r="AB8" s="58"/>
+      <c r="AC8" s="58"/>
+      <c r="AD8" s="58"/>
       <c r="AE8" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF8" s="50"/>
+        <v>49</v>
+      </c>
+      <c r="AF8" s="58"/>
       <c r="AG8" s="6"/>
     </row>
     <row r="9" spans="1:34" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="55" t="s">
+      <c r="A9" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="47" t="s">
+      <c r="B9" s="58"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="48"/>
+      <c r="F9" s="67"/>
       <c r="G9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="H9" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="J9" s="55" t="s">
+      <c r="J9" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="54"/>
-      <c r="N9" s="66" t="s">
+      <c r="K9" s="58"/>
+      <c r="L9" s="58"/>
+      <c r="M9" s="61"/>
+      <c r="N9" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="O9" s="50"/>
+      <c r="O9" s="58"/>
       <c r="P9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="Q9" s="67" t="s">
+      <c r="Q9" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="S9" s="55" t="s">
+      <c r="S9" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="T9" s="50"/>
-      <c r="U9" s="50"/>
+      <c r="T9" s="58"/>
+      <c r="U9" s="58"/>
       <c r="V9" s="62"/>
       <c r="W9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="X9" s="50"/>
+      <c r="X9" s="58"/>
       <c r="Y9" s="7"/>
       <c r="Z9" s="15"/>
-      <c r="AA9" s="55" t="s">
+      <c r="AA9" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="AB9" s="50"/>
-      <c r="AC9" s="50"/>
-      <c r="AD9" s="50"/>
+      <c r="AB9" s="58"/>
+      <c r="AC9" s="58"/>
+      <c r="AD9" s="58"/>
       <c r="AE9" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="AF9" s="50"/>
+      <c r="AF9" s="58"/>
       <c r="AG9" s="5"/>
     </row>
     <row r="10" spans="1:34" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="56"/>
-      <c r="B10" s="50"/>
-      <c r="C10" s="50"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="48"/>
+      <c r="A10" s="55"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="67"/>
       <c r="G10" s="43" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H10" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="J10" s="56"/>
-      <c r="K10" s="50"/>
-      <c r="L10" s="50"/>
-      <c r="M10" s="54"/>
+      <c r="J10" s="55"/>
+      <c r="K10" s="58"/>
+      <c r="L10" s="58"/>
+      <c r="M10" s="61"/>
       <c r="N10" s="42" t="s">
-        <v>67</v>
-      </c>
-      <c r="O10" s="50"/>
+        <v>66</v>
+      </c>
+      <c r="O10" s="58"/>
       <c r="P10" s="43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Q10" s="45" t="s">
-        <v>61</v>
-      </c>
-      <c r="S10" s="56"/>
-      <c r="T10" s="50"/>
-      <c r="U10" s="50"/>
+        <v>60</v>
+      </c>
+      <c r="S10" s="55"/>
+      <c r="T10" s="58"/>
+      <c r="U10" s="58"/>
       <c r="V10" s="63"/>
       <c r="W10" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="X10" s="50"/>
+        <v>47</v>
+      </c>
+      <c r="X10" s="58"/>
       <c r="Y10" s="8"/>
       <c r="Z10" s="16"/>
-      <c r="AA10" s="56"/>
-      <c r="AB10" s="50"/>
-      <c r="AC10" s="50"/>
-      <c r="AD10" s="50"/>
+      <c r="AA10" s="55"/>
+      <c r="AB10" s="58"/>
+      <c r="AC10" s="58"/>
+      <c r="AD10" s="58"/>
       <c r="AE10" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF10" s="50"/>
+        <v>50</v>
+      </c>
+      <c r="AF10" s="58"/>
       <c r="AG10" s="6"/>
     </row>
     <row r="11" spans="1:34" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="56" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="38" t="s">
@@ -2649,14 +2668,14 @@
       <c r="H11" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="52" t="s">
+      <c r="J11" s="69" t="s">
         <v>3</v>
       </c>
       <c r="K11" s="37" t="s">
         <v>10</v>
       </c>
       <c r="L11" s="39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M11" s="39" t="s">
         <v>13</v>
@@ -2669,7 +2688,7 @@
       <c r="Q11" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="S11" s="52" t="s">
+      <c r="S11" s="69" t="s">
         <v>3</v>
       </c>
       <c r="T11" s="39" t="s">
@@ -2685,7 +2704,7 @@
       <c r="X11" s="30"/>
       <c r="Y11" s="7"/>
       <c r="Z11" s="15"/>
-      <c r="AA11" s="52" t="s">
+      <c r="AA11" s="69" t="s">
         <v>3</v>
       </c>
       <c r="AB11" s="39" t="s">
@@ -2702,7 +2721,7 @@
       <c r="AG11" s="5"/>
     </row>
     <row r="12" spans="1:34" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="53"/>
+      <c r="A12" s="57"/>
       <c r="B12" s="41" t="s">
         <v>33</v>
       </c>
@@ -2715,17 +2734,17 @@
       <c r="E12" s="31"/>
       <c r="F12" s="32"/>
       <c r="G12" s="41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H12" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="J12" s="53"/>
+      <c r="J12" s="57"/>
       <c r="K12" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="L12" s="19" t="s">
         <v>62</v>
-      </c>
-      <c r="L12" s="19" t="s">
-        <v>63</v>
       </c>
       <c r="M12" s="41" t="s">
         <v>41</v>
@@ -2733,26 +2752,26 @@
       <c r="N12" s="31"/>
       <c r="O12" s="32"/>
       <c r="P12" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q12" s="44" t="s">
-        <v>59</v>
-      </c>
-      <c r="S12" s="53"/>
+        <v>58</v>
+      </c>
+      <c r="S12" s="57"/>
       <c r="T12" s="19" t="s">
         <v>25</v>
       </c>
       <c r="U12" s="41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V12" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="W12" s="31"/>
       <c r="X12" s="32"/>
       <c r="Y12" s="20"/>
       <c r="Z12" s="16"/>
-      <c r="AA12" s="53"/>
+      <c r="AA12" s="57"/>
       <c r="AB12" s="19" t="s">
         <v>24</v>
       </c>
@@ -2771,19 +2790,19 @@
       <c r="Z13" s="12"/>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A14" s="69"/>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69"/>
-      <c r="D14" s="69"/>
-      <c r="E14" s="69"/>
-      <c r="F14" s="69"/>
-      <c r="G14" s="69"/>
-      <c r="H14" s="69"/>
-      <c r="J14" s="68" t="s">
+      <c r="A14" s="65"/>
+      <c r="B14" s="65"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
+      <c r="J14" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="K14" s="49" t="s">
         <v>69</v>
-      </c>
-      <c r="K14" s="68" t="s">
-        <v>70</v>
       </c>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
@@ -2842,7 +2861,7 @@
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="J16" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K16" s="11">
         <v>15</v>
@@ -3154,6 +3173,85 @@
     </row>
   </sheetData>
   <mergeCells count="103">
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="AB9:AB10"/>
+    <mergeCell ref="AD3:AD4"/>
+    <mergeCell ref="AD5:AD6"/>
+    <mergeCell ref="AD7:AD8"/>
+    <mergeCell ref="AD9:AD10"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="AA11:AA12"/>
+    <mergeCell ref="S11:S12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="AF3:AF4"/>
+    <mergeCell ref="AF5:AF6"/>
+    <mergeCell ref="AF7:AF8"/>
+    <mergeCell ref="AF9:AF10"/>
+    <mergeCell ref="X3:X4"/>
+    <mergeCell ref="X5:X6"/>
+    <mergeCell ref="X7:X8"/>
+    <mergeCell ref="X9:X10"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="AA9:AA10"/>
+    <mergeCell ref="AC9:AC10"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="U7:U8"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="T5:T6"/>
+    <mergeCell ref="T7:T8"/>
+    <mergeCell ref="AA1:AC1"/>
+    <mergeCell ref="AE2:AF2"/>
+    <mergeCell ref="AA3:AA4"/>
+    <mergeCell ref="AC3:AC4"/>
+    <mergeCell ref="AB3:AB4"/>
+    <mergeCell ref="V5:V6"/>
+    <mergeCell ref="S7:S8"/>
+    <mergeCell ref="V7:V8"/>
+    <mergeCell ref="S9:S10"/>
+    <mergeCell ref="V9:V10"/>
+    <mergeCell ref="S1:U1"/>
+    <mergeCell ref="W2:X2"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="V3:V4"/>
+    <mergeCell ref="S5:S6"/>
+    <mergeCell ref="AB2:AC2"/>
+    <mergeCell ref="AA5:AA6"/>
+    <mergeCell ref="AC5:AC6"/>
+    <mergeCell ref="AA7:AA8"/>
+    <mergeCell ref="AC7:AC8"/>
+    <mergeCell ref="AB5:AB6"/>
+    <mergeCell ref="AB7:AB8"/>
+    <mergeCell ref="U9:U10"/>
+    <mergeCell ref="T9:T10"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="J1:L1"/>
     <mergeCell ref="N2:O2"/>
@@ -3178,88 +3276,9 @@
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M3:M4"/>
-    <mergeCell ref="AA1:AC1"/>
-    <mergeCell ref="AE2:AF2"/>
-    <mergeCell ref="AA3:AA4"/>
-    <mergeCell ref="AC3:AC4"/>
-    <mergeCell ref="AB3:AB4"/>
-    <mergeCell ref="V5:V6"/>
-    <mergeCell ref="S7:S8"/>
-    <mergeCell ref="V7:V8"/>
-    <mergeCell ref="S9:S10"/>
-    <mergeCell ref="V9:V10"/>
-    <mergeCell ref="S1:U1"/>
-    <mergeCell ref="W2:X2"/>
-    <mergeCell ref="S3:S4"/>
-    <mergeCell ref="V3:V4"/>
-    <mergeCell ref="S5:S6"/>
-    <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="AA5:AA6"/>
-    <mergeCell ref="AC5:AC6"/>
-    <mergeCell ref="AA7:AA8"/>
-    <mergeCell ref="AC7:AC8"/>
-    <mergeCell ref="AB5:AB6"/>
-    <mergeCell ref="AB7:AB8"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="U7:U8"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="T5:T6"/>
-    <mergeCell ref="T7:T8"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="AF3:AF4"/>
-    <mergeCell ref="AF5:AF6"/>
-    <mergeCell ref="AF7:AF8"/>
-    <mergeCell ref="AF9:AF10"/>
-    <mergeCell ref="X3:X4"/>
-    <mergeCell ref="X5:X6"/>
-    <mergeCell ref="X7:X8"/>
-    <mergeCell ref="X9:X10"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="O5:O6"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="AA9:AA10"/>
-    <mergeCell ref="AC9:AC10"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="AB9:AB10"/>
-    <mergeCell ref="AD3:AD4"/>
-    <mergeCell ref="AD5:AD6"/>
-    <mergeCell ref="AD7:AD8"/>
-    <mergeCell ref="AD9:AD10"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="AA11:AA12"/>
-    <mergeCell ref="S11:S12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="L9:L10"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>